<commit_message>
fixed data for 2026 measurements
</commit_message>
<xml_diff>
--- a/data/WRC Tree Measurements 2025.xlsx
+++ b/data/WRC Tree Measurements 2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailwsu.sharepoint.com/teams/cahnrs.treehealth/Shared Documents/Team Trees/Projects/Redcedar/Open Redcedar Adaptation Network/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailwsu-my.sharepoint.com/personal/zarina_gallardo_wsu_edu/Documents/Documents/GitHub/adaptation/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8280" documentId="13_ncr:1_{4869996F-A562-7344-B263-52C206E8DF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F96D3EB-9C72-43C4-8A22-08C410003799}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9F68BC5-A09D-4D5B-AF49-9FC0267331B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7550" yWindow="3390" windowWidth="28810" windowHeight="17410" activeTab="6" xr2:uid="{4396DE87-F012-D34B-8DBD-51148C600A68}"/>
+    <workbookView xWindow="-420" yWindow="2350" windowWidth="28810" windowHeight="17380" activeTab="6" xr2:uid="{4396DE87-F012-D34B-8DBD-51148C600A68}"/>
   </bookViews>
   <sheets>
     <sheet name="2022" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10180" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10164" uniqueCount="273">
   <si>
     <t>Tree Number</t>
   </si>
@@ -772,9 +772,6 @@
     <t>epicormic sprouting, minor flagging</t>
   </si>
   <si>
-    <t>flagging near base</t>
-  </si>
-  <si>
     <t>two dead trees nearby</t>
   </si>
   <si>
@@ -925,7 +922,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -960,8 +957,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -73015,14 +73010,14 @@
       <c r="E48" s="11">
         <v>46141</v>
       </c>
-      <c r="F48" s="9">
-        <v>109</v>
-      </c>
-      <c r="G48" s="9">
-        <v>19.100000000000001</v>
+      <c r="F48" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>204</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="I48" s="9"/>
       <c r="J48">
@@ -73531,7 +73526,7 @@
         <v>185</v>
       </c>
       <c r="G65">
-        <v>27.1</v>
+        <v>46.56</v>
       </c>
       <c r="H65" t="s">
         <v>27</v>
@@ -73679,7 +73674,7 @@
         <v>209</v>
       </c>
       <c r="G70">
-        <v>57.35</v>
+        <v>41.52</v>
       </c>
       <c r="H70" t="s">
         <v>27</v>
@@ -73707,7 +73702,7 @@
       <c r="F71">
         <v>153</v>
       </c>
-      <c r="G71" s="14">
+      <c r="G71">
         <v>32.07</v>
       </c>
       <c r="H71" t="s">
@@ -74305,7 +74300,7 @@
       </c>
     </row>
     <row r="91" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A91" s="15">
+      <c r="A91">
         <v>90</v>
       </c>
       <c r="B91" s="3">
@@ -74959,17 +74954,14 @@
       <c r="E112" s="11">
         <v>46143</v>
       </c>
-      <c r="F112">
-        <v>184</v>
-      </c>
-      <c r="G112">
-        <v>41.86</v>
-      </c>
-      <c r="H112" t="s">
-        <v>27</v>
-      </c>
-      <c r="I112" t="s">
-        <v>235</v>
+      <c r="F112" t="s">
+        <v>204</v>
+      </c>
+      <c r="G112" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="H112" s="3" t="s">
+        <v>29</v>
       </c>
       <c r="J112">
         <v>2026</v>
@@ -74992,16 +74984,16 @@
         <v>46143</v>
       </c>
       <c r="F113">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="G113">
-        <v>37.31</v>
+        <v>41.86</v>
       </c>
       <c r="H113" t="s">
         <v>27</v>
       </c>
       <c r="I113" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J113">
         <v>2026</v>
@@ -75027,10 +75019,13 @@
         <v>172</v>
       </c>
       <c r="G114">
-        <v>37.96</v>
+        <v>37.31</v>
       </c>
       <c r="H114" t="s">
         <v>27</v>
+      </c>
+      <c r="I114" t="s">
+        <v>236</v>
       </c>
       <c r="J114">
         <v>2026</v>
@@ -75053,10 +75048,10 @@
         <v>46143</v>
       </c>
       <c r="F115">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="G115">
-        <v>52.99</v>
+        <v>37.96</v>
       </c>
       <c r="H115" t="s">
         <v>27</v>
@@ -75082,16 +75077,13 @@
         <v>46143</v>
       </c>
       <c r="F116">
-        <v>216</v>
+        <v>196</v>
       </c>
       <c r="G116">
-        <v>60.08</v>
+        <v>52.99</v>
       </c>
       <c r="H116" t="s">
         <v>27</v>
-      </c>
-      <c r="I116" t="s">
-        <v>237</v>
       </c>
       <c r="J116">
         <v>2026</v>
@@ -75114,16 +75106,16 @@
         <v>46143</v>
       </c>
       <c r="F117">
-        <v>200</v>
+        <v>216</v>
       </c>
       <c r="G117">
-        <v>64.09</v>
+        <v>60.08</v>
       </c>
       <c r="H117" t="s">
         <v>27</v>
       </c>
       <c r="I117" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J117">
         <v>2026</v>
@@ -75146,13 +75138,16 @@
         <v>46143</v>
       </c>
       <c r="F118">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G118">
-        <v>55.02</v>
+        <v>64.09</v>
       </c>
       <c r="H118" t="s">
         <v>27</v>
+      </c>
+      <c r="I118" t="s">
+        <v>236</v>
       </c>
       <c r="J118">
         <v>2026</v>
@@ -75175,16 +75170,13 @@
         <v>46143</v>
       </c>
       <c r="F119">
-        <v>218</v>
+        <v>201</v>
       </c>
       <c r="G119">
-        <v>70.09</v>
+        <v>55.02</v>
       </c>
       <c r="H119" t="s">
         <v>27</v>
-      </c>
-      <c r="I119" t="s">
-        <v>238</v>
       </c>
       <c r="J119">
         <v>2026</v>
@@ -75207,16 +75199,16 @@
         <v>46143</v>
       </c>
       <c r="F120">
-        <v>196</v>
+        <v>218</v>
       </c>
       <c r="G120">
-        <v>51.33</v>
+        <v>70.09</v>
       </c>
       <c r="H120" t="s">
         <v>27</v>
       </c>
       <c r="I120" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="J120">
         <v>2026</v>
@@ -75239,16 +75231,16 @@
         <v>46143</v>
       </c>
       <c r="F121">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="G121">
-        <v>50.22</v>
+        <v>51.33</v>
       </c>
       <c r="H121" t="s">
         <v>27</v>
       </c>
       <c r="I121" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="J121">
         <v>2026</v>
@@ -75271,10 +75263,10 @@
         <v>46143</v>
       </c>
       <c r="F122">
-        <v>269</v>
+        <v>217</v>
       </c>
       <c r="G122">
-        <v>54.95</v>
+        <v>50.22</v>
       </c>
       <c r="H122" t="s">
         <v>27</v>
@@ -75303,13 +75295,16 @@
         <v>46143</v>
       </c>
       <c r="F123">
-        <v>190</v>
+        <v>269</v>
       </c>
       <c r="G123">
-        <v>43.34</v>
+        <v>54.95</v>
       </c>
       <c r="H123" t="s">
         <v>27</v>
+      </c>
+      <c r="I123" t="s">
+        <v>223</v>
       </c>
       <c r="J123">
         <v>2026</v>
@@ -75332,10 +75327,10 @@
         <v>46143</v>
       </c>
       <c r="F124">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="G124">
-        <v>33.51</v>
+        <v>43.34</v>
       </c>
       <c r="H124" t="s">
         <v>27</v>
@@ -75361,10 +75356,10 @@
         <v>46143</v>
       </c>
       <c r="F125">
-        <v>160</v>
+        <v>183</v>
       </c>
       <c r="G125">
-        <v>33.44</v>
+        <v>33.51</v>
       </c>
       <c r="H125" t="s">
         <v>27</v>
@@ -75390,10 +75385,10 @@
         <v>46143</v>
       </c>
       <c r="F126">
-        <v>173</v>
+        <v>160</v>
       </c>
       <c r="G126">
-        <v>45.32</v>
+        <v>33.44</v>
       </c>
       <c r="H126" t="s">
         <v>27</v>
@@ -75419,10 +75414,10 @@
         <v>46143</v>
       </c>
       <c r="F127">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="G127">
-        <v>49.93</v>
+        <v>45.32</v>
       </c>
       <c r="H127" t="s">
         <v>27</v>
@@ -75448,10 +75443,10 @@
         <v>46143</v>
       </c>
       <c r="F128">
-        <v>213</v>
+        <v>186</v>
       </c>
       <c r="G128">
-        <v>49.45</v>
+        <v>49.93</v>
       </c>
       <c r="H128" t="s">
         <v>27</v>
@@ -75477,10 +75472,10 @@
         <v>46143</v>
       </c>
       <c r="F129">
-        <v>186</v>
+        <v>213</v>
       </c>
       <c r="G129">
-        <v>47.88</v>
+        <v>49.45</v>
       </c>
       <c r="H129" t="s">
         <v>27</v>
@@ -75506,10 +75501,10 @@
         <v>46143</v>
       </c>
       <c r="F130">
-        <v>238</v>
+        <v>186</v>
       </c>
       <c r="G130">
-        <v>51.73</v>
+        <v>47.88</v>
       </c>
       <c r="H130" t="s">
         <v>27</v>
@@ -75535,16 +75530,13 @@
         <v>46143</v>
       </c>
       <c r="F131">
-        <v>203</v>
+        <v>238</v>
       </c>
       <c r="G131">
-        <v>51.11</v>
+        <v>51.73</v>
       </c>
       <c r="H131" t="s">
         <v>27</v>
-      </c>
-      <c r="I131" t="s">
-        <v>234</v>
       </c>
       <c r="J131">
         <v>2026</v>
@@ -75567,13 +75559,16 @@
         <v>46143</v>
       </c>
       <c r="F132">
-        <v>216</v>
+        <v>203</v>
       </c>
       <c r="G132">
-        <v>54.21</v>
+        <v>51.11</v>
       </c>
       <c r="H132" t="s">
         <v>27</v>
+      </c>
+      <c r="I132" t="s">
+        <v>234</v>
       </c>
       <c r="J132">
         <v>2026</v>
@@ -75596,10 +75591,10 @@
         <v>46143</v>
       </c>
       <c r="F133">
-        <v>255</v>
+        <v>216</v>
       </c>
       <c r="G133">
-        <v>56.62</v>
+        <v>54.21</v>
       </c>
       <c r="H133" t="s">
         <v>27</v>
@@ -75625,10 +75620,10 @@
         <v>46143</v>
       </c>
       <c r="F134">
-        <v>209</v>
+        <v>255</v>
       </c>
       <c r="G134">
-        <v>48.11</v>
+        <v>56.62</v>
       </c>
       <c r="H134" t="s">
         <v>27</v>
@@ -75654,10 +75649,10 @@
         <v>46143</v>
       </c>
       <c r="F135">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="G135">
-        <v>46.73</v>
+        <v>48.11</v>
       </c>
       <c r="H135" t="s">
         <v>27</v>
@@ -75683,16 +75678,13 @@
         <v>46143</v>
       </c>
       <c r="F136">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="G136">
-        <v>51.1</v>
+        <v>46.73</v>
       </c>
       <c r="H136" t="s">
         <v>27</v>
-      </c>
-      <c r="I136" t="s">
-        <v>228</v>
       </c>
       <c r="J136">
         <v>2026</v>
@@ -75715,16 +75707,16 @@
         <v>46143</v>
       </c>
       <c r="F137">
-        <v>232</v>
+        <v>185</v>
       </c>
       <c r="G137">
-        <v>43.61</v>
+        <v>51.1</v>
       </c>
       <c r="H137" t="s">
         <v>27</v>
       </c>
       <c r="I137" t="s">
-        <v>112</v>
+        <v>228</v>
       </c>
       <c r="J137">
         <v>2026</v>
@@ -75747,16 +75739,16 @@
         <v>46143</v>
       </c>
       <c r="F138">
-        <v>179</v>
+        <v>232</v>
       </c>
       <c r="G138">
-        <v>41.72</v>
+        <v>43.61</v>
       </c>
       <c r="H138" t="s">
         <v>27</v>
       </c>
       <c r="I138" t="s">
-        <v>223</v>
+        <v>112</v>
       </c>
       <c r="J138">
         <v>2026</v>
@@ -75779,16 +75771,16 @@
         <v>46143</v>
       </c>
       <c r="F139">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G139">
-        <v>39.479999999999997</v>
+        <v>41.72</v>
       </c>
       <c r="H139" t="s">
         <v>27</v>
       </c>
       <c r="I139" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="J139">
         <v>2026</v>
@@ -75811,10 +75803,10 @@
         <v>46143</v>
       </c>
       <c r="F140">
-        <v>206</v>
+        <v>177</v>
       </c>
       <c r="G140">
-        <v>46.82</v>
+        <v>39.479999999999997</v>
       </c>
       <c r="H140" t="s">
         <v>27</v>
@@ -75843,16 +75835,16 @@
         <v>46143</v>
       </c>
       <c r="F141">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G141">
-        <v>53.96</v>
+        <v>46.82</v>
       </c>
       <c r="H141" t="s">
         <v>27</v>
       </c>
       <c r="I141" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="J141">
         <v>2026</v>
@@ -75875,13 +75867,16 @@
         <v>46143</v>
       </c>
       <c r="F142">
-        <v>279</v>
+        <v>212</v>
       </c>
       <c r="G142">
-        <v>71.13</v>
+        <v>53.96</v>
       </c>
       <c r="H142" t="s">
         <v>27</v>
+      </c>
+      <c r="I142" t="s">
+        <v>239</v>
       </c>
       <c r="J142">
         <v>2026</v>
@@ -75904,10 +75899,10 @@
         <v>46143</v>
       </c>
       <c r="F143">
-        <v>171</v>
+        <v>279</v>
       </c>
       <c r="G143">
-        <v>34.6</v>
+        <v>71.13</v>
       </c>
       <c r="H143" t="s">
         <v>27</v>
@@ -75941,9 +75936,6 @@
       <c r="H144" t="s">
         <v>27</v>
       </c>
-      <c r="I144" t="s">
-        <v>219</v>
-      </c>
       <c r="J144">
         <v>2026</v>
       </c>
@@ -75973,6 +75965,9 @@
       <c r="H145" t="s">
         <v>32</v>
       </c>
+      <c r="I145" t="s">
+        <v>219</v>
+      </c>
       <c r="J145">
         <v>2026</v>
       </c>
@@ -76002,9 +75997,6 @@
       <c r="H146" t="s">
         <v>27</v>
       </c>
-      <c r="I146" t="s">
-        <v>240</v>
-      </c>
       <c r="J146">
         <v>2026</v>
       </c>
@@ -76064,7 +76056,7 @@
         <v>27</v>
       </c>
       <c r="I148" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="J148">
         <v>2026</v>
@@ -76125,7 +76117,7 @@
         <v>27</v>
       </c>
       <c r="I150" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="J150">
         <v>2026</v>
@@ -76334,7 +76326,7 @@
         <v>27</v>
       </c>
       <c r="I157" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="J157">
         <v>2026</v>
@@ -76366,7 +76358,7 @@
         <v>27</v>
       </c>
       <c r="I158" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J158">
         <v>2026</v>
@@ -76430,7 +76422,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="161" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A161">
         <v>160</v>
       </c>
@@ -76459,7 +76451,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="162" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>161</v>
       </c>
@@ -76485,13 +76477,13 @@
         <v>27</v>
       </c>
       <c r="I162" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J162">
         <v>2026</v>
       </c>
     </row>
-    <row r="163" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>162</v>
       </c>
@@ -76523,7 +76515,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="164" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>163</v>
       </c>
@@ -76552,7 +76544,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="165" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>164</v>
       </c>
@@ -76581,7 +76573,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="166" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A166">
         <v>165</v>
       </c>
@@ -76607,13 +76599,13 @@
         <v>27</v>
       </c>
       <c r="I166" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J166">
         <v>2026</v>
       </c>
     </row>
-    <row r="167" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A167">
         <v>166</v>
       </c>
@@ -76639,13 +76631,13 @@
         <v>27</v>
       </c>
       <c r="I167" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="J167">
         <v>2026</v>
       </c>
     </row>
-    <row r="168" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>167</v>
       </c>
@@ -76674,7 +76666,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="169" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A169">
         <v>168</v>
       </c>
@@ -76700,13 +76692,13 @@
         <v>27</v>
       </c>
       <c r="I169" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="J169">
         <v>2026</v>
       </c>
     </row>
-    <row r="170" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A170">
         <v>169</v>
       </c>
@@ -76735,7 +76727,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="171" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A171">
         <v>170</v>
       </c>
@@ -76761,16 +76753,13 @@
         <v>27</v>
       </c>
       <c r="I171" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J171">
         <v>2026</v>
       </c>
-      <c r="K171" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="172" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="172" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A172">
         <v>171</v>
       </c>
@@ -76799,7 +76788,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="173" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A173">
         <v>172</v>
       </c>
@@ -76831,7 +76820,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="174" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A174">
         <v>173</v>
       </c>
@@ -76857,16 +76846,13 @@
         <v>27</v>
       </c>
       <c r="I174" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J174">
         <v>2026</v>
       </c>
-      <c r="K174" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="175" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="175" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>174</v>
       </c>
@@ -76895,7 +76881,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="176" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A176">
         <v>175</v>
       </c>
@@ -76924,7 +76910,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="177" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A177">
         <v>176</v>
       </c>
@@ -76953,7 +76939,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="178" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>177</v>
       </c>
@@ -76979,16 +76965,13 @@
         <v>27</v>
       </c>
       <c r="I178" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="J178">
         <v>2026</v>
       </c>
-      <c r="K178" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="179" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="179" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A179">
         <v>178</v>
       </c>
@@ -77014,13 +76997,13 @@
         <v>27</v>
       </c>
       <c r="I179" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="J179">
         <v>2026</v>
       </c>
     </row>
-    <row r="180" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>179</v>
       </c>
@@ -77046,16 +77029,13 @@
         <v>27</v>
       </c>
       <c r="I180" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J180">
         <v>2026</v>
       </c>
-      <c r="K180" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="181" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="181" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>180</v>
       </c>
@@ -77084,7 +77064,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="182" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A182">
         <v>181</v>
       </c>
@@ -77113,7 +77093,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="183" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A183">
         <v>182</v>
       </c>
@@ -77139,16 +77119,13 @@
         <v>27</v>
       </c>
       <c r="I183" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J183">
         <v>2026</v>
       </c>
-      <c r="K183" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="184" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="184" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>183</v>
       </c>
@@ -77174,16 +77151,13 @@
         <v>27</v>
       </c>
       <c r="I184" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J184">
         <v>2026</v>
       </c>
-      <c r="K184" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="185" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="185" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>184</v>
       </c>
@@ -77209,13 +77183,13 @@
         <v>32</v>
       </c>
       <c r="I185" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="J185">
         <v>2026</v>
       </c>
     </row>
-    <row r="186" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A186">
         <v>185</v>
       </c>
@@ -77247,7 +77221,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="187" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A187">
         <v>186</v>
       </c>
@@ -77276,7 +77250,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="188" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>187</v>
       </c>
@@ -77305,7 +77279,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="189" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A189">
         <v>188</v>
       </c>
@@ -77331,13 +77305,13 @@
         <v>32</v>
       </c>
       <c r="I189" s="3" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J189">
         <v>2026</v>
       </c>
     </row>
-    <row r="190" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A190">
         <v>189</v>
       </c>
@@ -77369,7 +77343,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="191" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A191">
         <v>190</v>
       </c>
@@ -77398,7 +77372,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="192" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>191</v>
       </c>
@@ -77424,13 +77398,13 @@
         <v>32</v>
       </c>
       <c r="I192" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="J192">
         <v>2026</v>
       </c>
     </row>
-    <row r="193" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>192</v>
       </c>
@@ -77459,7 +77433,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="194" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A194">
         <v>193</v>
       </c>
@@ -77488,7 +77462,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="195" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>194</v>
       </c>
@@ -77514,16 +77488,13 @@
         <v>27</v>
       </c>
       <c r="I195" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J195">
         <v>2026</v>
       </c>
-      <c r="K195" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="196" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="196" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>195</v>
       </c>
@@ -77552,7 +77523,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="197" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>196</v>
       </c>
@@ -77578,16 +77549,13 @@
         <v>27</v>
       </c>
       <c r="I197" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J197">
         <v>2026</v>
       </c>
-      <c r="K197" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="198" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="198" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A198">
         <v>197</v>
       </c>
@@ -77616,7 +77584,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="199" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A199">
         <v>198</v>
       </c>
@@ -77645,7 +77613,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="200" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A200">
         <v>199</v>
       </c>
@@ -77671,13 +77639,13 @@
         <v>27</v>
       </c>
       <c r="I200" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J200">
         <v>2026</v>
       </c>
     </row>
-    <row r="201" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A201">
         <v>200</v>
       </c>
@@ -77703,16 +77671,13 @@
         <v>27</v>
       </c>
       <c r="I201" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J201">
         <v>2026</v>
       </c>
-      <c r="K201" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="202" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="202" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A202">
         <v>201</v>
       </c>
@@ -77738,13 +77703,13 @@
         <v>27</v>
       </c>
       <c r="I202" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J202">
         <v>2026</v>
       </c>
     </row>
-    <row r="203" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A203">
         <v>202</v>
       </c>
@@ -77773,7 +77738,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="204" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A204">
         <v>203</v>
       </c>
@@ -77805,7 +77770,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="205" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A205">
         <v>204</v>
       </c>
@@ -77831,16 +77796,13 @@
         <v>27</v>
       </c>
       <c r="I205" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J205">
         <v>2026</v>
       </c>
-      <c r="K205" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="206" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="206" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A206">
         <v>205</v>
       </c>
@@ -77872,7 +77834,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="207" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A207">
         <v>206</v>
       </c>
@@ -77904,7 +77866,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="208" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A208">
         <v>207</v>
       </c>
@@ -77930,16 +77892,13 @@
         <v>27</v>
       </c>
       <c r="I208" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J208">
         <v>2026</v>
       </c>
-      <c r="K208" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="209" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="209" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A209">
         <v>208</v>
       </c>
@@ -77968,7 +77927,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="210" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A210">
         <v>209</v>
       </c>
@@ -78000,7 +77959,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="211" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A211">
         <v>210</v>
       </c>
@@ -78029,7 +77988,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="212" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A212">
         <v>211</v>
       </c>
@@ -78055,16 +78014,13 @@
         <v>27</v>
       </c>
       <c r="I212" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J212">
         <v>2026</v>
       </c>
-      <c r="K212" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="213" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="213" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A213">
         <v>212</v>
       </c>
@@ -78093,7 +78049,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="214" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A214">
         <v>213</v>
       </c>
@@ -78119,13 +78075,13 @@
         <v>27</v>
       </c>
       <c r="I214" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J214">
         <v>2026</v>
       </c>
     </row>
-    <row r="215" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A215">
         <v>214</v>
       </c>
@@ -78151,16 +78107,13 @@
         <v>27</v>
       </c>
       <c r="I215" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J215">
         <v>2026</v>
       </c>
-      <c r="K215" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="216" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="216" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A216">
         <v>215</v>
       </c>
@@ -78186,13 +78139,13 @@
         <v>27</v>
       </c>
       <c r="I216" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J216">
         <v>2026</v>
       </c>
     </row>
-    <row r="217" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A217">
         <v>216</v>
       </c>
@@ -78218,13 +78171,13 @@
         <v>27</v>
       </c>
       <c r="I217" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J217">
         <v>2026</v>
       </c>
     </row>
-    <row r="218" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A218">
         <v>217</v>
       </c>
@@ -78253,7 +78206,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="219" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A219">
         <v>218</v>
       </c>
@@ -78279,16 +78232,13 @@
         <v>27</v>
       </c>
       <c r="I219" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J219">
         <v>2026</v>
       </c>
-      <c r="K219" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="220" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="220" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A220">
         <v>219</v>
       </c>
@@ -78314,16 +78264,13 @@
         <v>27</v>
       </c>
       <c r="I220" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J220">
         <v>2026</v>
       </c>
-      <c r="K220" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="221" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="221" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A221">
         <v>220</v>
       </c>
@@ -78349,16 +78296,13 @@
         <v>27</v>
       </c>
       <c r="I221" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J221">
         <v>2026</v>
       </c>
-      <c r="K221" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="222" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="222" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A222">
         <v>221</v>
       </c>
@@ -78390,7 +78334,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="223" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A223">
         <v>222</v>
       </c>
@@ -78416,16 +78360,13 @@
         <v>27</v>
       </c>
       <c r="I223" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J223">
         <v>2026</v>
       </c>
-      <c r="K223" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="224" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="224" spans="1:10" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A224">
         <v>223</v>
       </c>
@@ -78451,7 +78392,7 @@
         <v>27</v>
       </c>
       <c r="I224" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="J224">
         <v>2026</v>
@@ -78483,7 +78424,7 @@
         <v>27</v>
       </c>
       <c r="I225" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J225">
         <v>2026</v>
@@ -78515,7 +78456,7 @@
         <v>27</v>
       </c>
       <c r="I226" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="J226">
         <v>2026</v>
@@ -78663,13 +78604,10 @@
         <v>27</v>
       </c>
       <c r="I231" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="J231">
         <v>2026</v>
-      </c>
-      <c r="K231" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="232" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
@@ -78727,7 +78665,7 @@
         <v>27</v>
       </c>
       <c r="I233" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J233">
         <v>2026</v>
@@ -78759,7 +78697,7 @@
         <v>27</v>
       </c>
       <c r="I234" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="J234">
         <v>2026</v>
@@ -78791,7 +78729,7 @@
         <v>27</v>
       </c>
       <c r="I235" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J235">
         <v>2026</v>
@@ -78852,13 +78790,10 @@
         <v>27</v>
       </c>
       <c r="I237" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J237">
         <v>2026</v>
-      </c>
-      <c r="K237" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="238" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
@@ -78931,9 +78866,6 @@
       </c>
       <c r="D240" t="s">
         <v>12</v>
-      </c>
-      <c r="J240">
-        <v>2026</v>
       </c>
       <c r="K240" t="s">
         <v>130</v>
@@ -81401,18 +81333,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="56ba983a-c5de-4d8d-8995-cdf23a31bf22">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0fcbb840-36bc-46d8-9c5c-6ccae2a4d649" xsi:nil="true"/>
-    <Sample xmlns="56ba983a-c5de-4d8d-8995-cdf23a31bf22" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E04F2B8CC697774992AE10D6F9880B5C" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c6291a289f0bb36b1209bde0e204f480">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="56ba983a-c5de-4d8d-8995-cdf23a31bf22" xmlns:ns3="0fcbb840-36bc-46d8-9c5c-6ccae2a4d649" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e01a86dd7d84021e8c471956e4d1d876" ns2:_="" ns3:_="">
     <xsd:import namespace="56ba983a-c5de-4d8d-8995-cdf23a31bf22"/>
@@ -81661,6 +81581,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="56ba983a-c5de-4d8d-8995-cdf23a31bf22">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0fcbb840-36bc-46d8-9c5c-6ccae2a4d649" xsi:nil="true"/>
+    <Sample xmlns="56ba983a-c5de-4d8d-8995-cdf23a31bf22" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{123DEC97-4516-4AC2-8F6D-0FD2A41D3DFC}">
   <ds:schemaRefs>
@@ -81670,22 +81602,37 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51079DBE-67B3-454B-B314-CB1705B12DE3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD752820-E061-4F17-8DE4-DE0BA715D3F4}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="56ba983a-c5de-4d8d-8995-cdf23a31bf22"/>
+    <ds:schemaRef ds:uri="0fcbb840-36bc-46d8-9c5c-6ccae2a4d649"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0fcbb840-36bc-46d8-9c5c-6ccae2a4d649"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="56ba983a-c5de-4d8d-8995-cdf23a31bf22"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD752820-E061-4F17-8DE4-DE0BA715D3F4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{51079DBE-67B3-454B-B314-CB1705B12DE3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0fcbb840-36bc-46d8-9c5c-6ccae2a4d649"/>
+    <ds:schemaRef ds:uri="56ba983a-c5de-4d8d-8995-cdf23a31bf22"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>